<commit_message>
feat: all translation correciton and merge
</commit_message>
<xml_diff>
--- a/data_extactor/batch_10_fa/batch_0001_fa.xlsx
+++ b/data_extactor/batch_10_fa/batch_0001_fa.xlsx
@@ -503,32 +503,32 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AdSense Tracker | Adobe Acrobat | Atlassian JIRA | Blackbaud The Raiser's Edge | نرم‌افزار حسابداری ساخت و ساز ComputerEase | نرم‌افزار گزارش‌گیری پایگاه داده | Databox | نرم‌افزار ایمیل | Exact Software Macola ES Labor Performance | زبان نشانه‌گذاری توسعه‌پذیر XML | نرم‌افزار حسابداری صندوق | نرم‌افزار ارائه گرافیکی | HCSS HeavyBid | HCSS HeavyJob | Halogen e360 | Halogen ePraisal | سیستم اطلاعات منابع انسانی (HRIS) | Infor SSA Human Capital Management | Intuit QuickBooks | نرم‌افزار Listserv | Lyris HQ Web-Analytics Solution | Mentimeter | Microsoft Access | Microsoft Dynamics | Microsoft Dynamics AX | Microsoft Dynamics GP | Microsoft Excel | Microsoft FRx | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SharePoint | Microsoft Word | Nedstat Sitestat | Norchard Solutions Succession Wizard | نرم‌افزار گزارش‌گیری تبلیغات آنلاین | Oracle E-Business Suite | Oracle PeopleSoft | Oracle Siebel Server Sync | PHP | نرم‌افزار مدیریت پایگاه داده رابطه‌ای | نرم‌افزار SAP | Sage 50 Accounting | SmugMug Flickr | زبان پرس و جوی ساختاریافته SQL | نرم‌افزار مرورگر وب</t>
+          <t>AdSense Tracker | Adobe Acrobat | Atlassian JIRA | Blackbaud The Raiser's Edge | نرم‌افزار حسابداری ساخت‌وساز ComputerEase | نرم‌افزار گزارش‌گیری پایگاه داده | Databox | نرم‌افزار ایمیل | Exact Software Macola ES Labor Performance | زبان نشانه‌گذاری توسعه‌پذیر XML | نرم‌افزار حسابداری صندوق | نرم‌افزار ارائه گرافیکی | HCSS HeavyBid | HCSS HeavyJob | Halogen e360 | Halogen ePraisal | سیستم اطلاعات منابع انسانی (HRIS) | Infor SSA Human Capital Management | Intuit QuickBooks | نرم‌افزار Listserv | Lyris HQ Web-Analytics Solution | Mentimeter | Microsoft Access | Microsoft Dynamics | Microsoft Dynamics AX | Microsoft Dynamics GP | Microsoft Excel | Microsoft FRx | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SharePoint | Microsoft Word | Nedstat Sitestat | Norchard Solutions Succession Wizard | نرم‌افزار گزارش‌گیری تبلیغات آنلاین | Oracle E-Business Suite | Oracle PeopleSoft | Oracle Siebel Server Sync | PHP | نرم‌افزار مدیریت پایگاه داده رابطه‌ای | نرم‌افزار SAP | Sage 50 Accounting | SmugMug Flickr | زبان پرس‌وجوی ساختاریافته SQL | نرم‌افزار مرورگر وب</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>تفکر انتقادی | صحبت کردن | درک مطلب | نوشتن | گوش دادن فعال | نظارت | یادگیری فعال | ریاضیات | استراتژی‌های یادگیری</t>
+          <t>تفکر انتقادی | سخن گفتن | درک مطلب | نگارش | گوش دادن فعال | نظارت | یادگیری فعال | ریاضیات | راهبردهای یادگیری</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>مدیریت و اداره | پرسنل و منابع انسانی | زبان انگلیسی | خدمات مشتری و شخصی | اقتصاد و حسابداری | ایمنی و امنیت عمومی | رایانه‌ها و الکترونیک | فروش و بازاریابی | ریاضیات | آموزش و تعلیم | قانون و دولت | روانشناسی | مهندسی و فناوری | ارتباطات و رسانه</t>
+          <t>مدیریت و اداره | پرسنل و منابع انسانی | زبان انگلیسی | خدمات مشتری و شخصی | اقتصاد و حسابداری | ایمنی و امنیت عمومی | رایانه و الکترونیک | فروش و بازاریابی | ریاضیات | آموزش و پرورش | قانون و دولت | روان‌شناسی | مهندسی و فناوری | ارتباطات و رسانه</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>درک شفاهی | بیان شفاهی | درک کتبی | وضوح گفتار | بیان کتبی | استدلال قیاسی | تشخیص گفتار | مرتب‌سازی اطلاعات | استدلال استقرایی | حساسیت به مشکل | روانی ایده‌ها | اصالت | بینایی نزدیک | انعطاف‌پذیری دسته‌بندی | استدلال ریاضی | انعطاف‌پذیری انسداد | سهولت در اعداد | سرعت ادراکی | بینایی دور | توجه انتخابی | تجسم | سرعت انسداد</t>
+          <t>درک شفاهی | بیان شفاهی | درک کتبی | وضوح گفتار | بیان کتبی | استدلال قیاسی | تشخیص گفتار | ترتیب‌دهی اطلاعات | استدلال استقرایی | حساسیت به مسئله | روانی ایده‌ها | اصالت | بینایی نزدیک | انعطاف‌پذیری دسته‌بندی | استدلال ریاضی | انعطاف‌پذیری بستار | توانایی عددی | سرعت ادراکی | بینایی دور | توجه انتخابی | تجسم | سرعت بستار</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ایمیل | آزادی در تصمیم‌گیری | مکالمات تلفنی | بحث‌های چهره به چهره با افراد و درون تیم‌ها | فضای داخلی، با محیط کنترل‌شده | تعیین وظایف، اولویت‌ها و اهداف | تأثیر تصمیمات بر همکاران یا نتایج شرکت | پیامدهای کاری و نتایج سایر کارگران | فرکانس تصمیم‌گیری | تماس با دیگران | اهمیت دقیق یا صحیح بودن | کار با یا مشارکت در یک گروه کاری یا تیم | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | صرف زمان برای نشستن | بهداشت و ایمنی سایر کارگران | فشار زمانی | نامه‌ها و یادداشت‌های کتبی | موقعیت‌های تعارض | سطح رقابت</t>
+          <t>ایمیل | آزادی در تصمیم‌گیری | مکالمات تلفنی | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | محیط داخلی، دارای کنترل شرایط محیطی | تعیین وظایف، اولویت‌ها و اهداف | تأثیر تصمیمات بر همکاران یا نتایج شرکت | پیامدهای کاری و نتایج سایر کارکنان | فراوانی تصمیم‌گیری | ارتباط با دیگران | اهمیت دقیق یا درست بودن | کار با یا مشارکت در یک گروه کاری یا تیم | تعامل با مشتریان خارجی یا عموم مردم | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | صرف زمان برای نشستن | سلامت و ایمنی سایر کارکنان | فشار زمانی | نامه‌ها و یادداشت‌های کتبی | موقعیت‌های تعارض | سطح رقابت</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>مدیران خدمات اداری | مدیران ارشد پایداری | مدیران انطباق | مدیران آموزش، پس از متوسطه | منشی‌های اجرایی و دستیاران اداری اجرایی | بازرسان مالی | مدیران مالی | سرپرستان خط اول کارگران فروش غیر خرده‌فروشی | سرپرستان خط اول کارگران پشتیبانی اداری و دفتری | مدیران عمومی و عملیات | مدیران منابع انسانی | متخصصان روابط کار | قانون‌گذاران | تحلیل‌گران مدیریت | مدیران روابط عمومی | متخصصان روابط عمومی | مدیران فروش | منشی‌ها و دستیاران اداری، به استثنای حقوقی، پزشکی و اجرایی | مدیران خدمات اجتماعی و جامعه | خزانه‌داران و کنترل‌کننده‌ها</t>
+          <t>مدیران خدمات اداری | مدیران ارشد پایداری | مدیران انطباق | مدیران آموزشی، پس از متوسطه | منشی‌های اجرایی و دستیاران اداری اجرایی | بازرسان مالی | مدیران مالی | سرپرستان رده اول کارکنان فروش غیرخرده‌فروشی | سرپرستان خط اول کارکنان دفتری و پشتیبانی اداری | مدیران عمومی و عملیات | مدیران منابع انسانی | متخصصان روابط کار | قانون‌گذاران | تحلیل‌گران مدیریت | مدیران روابط عمومی | متخصصان روابط عمومی | مدیران فروش | منشی‌ها و دستیاران اداری، به جز حقوقی، پزشکی و اجرایی | مدیران خدمات اجتماعی و جامعه | خزانه‌داران و کنترل‌کنندگان</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -560,32 +560,32 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Adobe Acrobat | Adobe Photoshop | نرم‌افزار ایمیل | Facebook | سیستم‌های اطلاعات مدیریت MIS | Microsoft Access | Microsoft Dynamics GP | Microsoft Excel | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft SharePoint | Microsoft Word | نرم‌افزار SAP | نرم‌افزار Salesforce | نرم‌افزار زمان‌بندی | زبان پرس و جوی ساختاریافته SQL | Tableau | نرم‌افزار کنفرانس از راه دور | نرم‌افزار مرورگر وب</t>
+          <t>Adobe Acrobat | Adobe Photoshop | نرم‌افزار ایمیل | Facebook | سیستم‌های اطلاعات مدیریت MIS | Microsoft Access | Microsoft Dynamics GP | Microsoft Excel | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft SharePoint | Microsoft Word | نرم‌افزار SAP | نرم‌افزار Salesforce | نرم‌افزار زمان‌بندی | زبان پرس‌وجوی ساختاریافته SQL | Tableau | نرم‌افزار کنفرانس از راه دور | نرم‌افزار مرورگر وب</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>نوشتن | تفکر انتقادی | صحبت کردن | گوش دادن فعال | درک مطلب | نظارت | یادگیری فعال | استراتژی‌های یادگیری</t>
+          <t>نگارش | تفکر انتقادی | سخن گفتن | گوش دادن فعال | درک مطلب | نظارت | یادگیری فعال | راهبردهای یادگیری</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>زبان انگلیسی | مدیریت و اداره | قانون و دولت | ارتباطات و رسانه | ساختمان و ساخت و ساز | خدمات مشتری و شخصی | آموزش و تعلیم | اقتصاد و حسابداری | فروش و بازاریابی | حمل و نقل | جغرافیا | جامعه‌شناسی و انسان‌شناسی | پرسنل و منابع انسانی | ریاضیات</t>
+          <t>زبان انگلیسی | مدیریت و اداره | قانون و دولت | ارتباطات و رسانه | ساختمان و ساخت‌وساز | خدمات مشتری و شخصی | آموزش و پرورش | اقتصاد و حسابداری | فروش و بازاریابی | حمل و نقل | جغرافیا | جامعه‌شناسی و انسان‌شناسی | پرسنل و منابع انسانی | ریاضیات</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>بیان کتبی | درک شفاهی | درک کتبی | بیان شفاهی | تشخیص گفتار | وضوح گفتار | حساسیت به مشکل | استدلال قیاسی | استدلال استقرایی | روانی ایده‌ها | اصالت | مرتب‌سازی اطلاعات | بینایی نزدیک | توجه انتخابی | انعطاف‌پذیری دسته‌بندی</t>
+          <t>بیان کتبی | درک شفاهی | درک کتبی | بیان شفاهی | تشخیص گفتار | وضوح گفتار | حساسیت به مسئله | استدلال قیاسی | استدلال استقرایی | روانی ایده‌ها | اصالت | ترتیب‌دهی اطلاعات | بینایی نزدیک | توجه انتخابی | انعطاف‌پذیری دسته‌بندی</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ایمیل | کار با یا مشارکت در یک گروه کاری یا تیم | فضای داخلی، با محیط کنترل‌شده | مکالمات تلفنی | بحث‌های چهره به چهره با افراد و درون تیم‌ها | تعیین وظایف، اولویت‌ها و اهداف | تماس با دیگران | آزادی در تصمیم‌گیری | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | صرف زمان برای نشستن | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | پیامدهای کاری و نتایج سایر کارگران | سطح رقابت | فرکانس تصمیم‌گیری | اهمیت دقیق یا صحیح بودن</t>
+          <t>ایمیل | کار با یا مشارکت در یک گروه کاری یا تیم | محیط داخلی، دارای کنترل شرایط محیطی | مکالمات تلفنی | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | تعیین وظایف، اولویت‌ها و اهداف | ارتباط با دیگران | آزادی در تصمیم‌گیری | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | صرف زمان برای نشستن | تعامل با مشتریان خارجی یا عموم مردم | پیامدهای کاری و نتایج سایر کارکنان | سطح رقابت | فراوانی تصمیم‌گیری | اهمیت دقیق یا درست بودن</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>متخصصان توسعه مجدد زمین‌های قهوه‌ای و مدیران سایت | مدیران ارشد اجرایی | تحلیل‌گران سیاست تغییرات آب و هوایی | مدیران انطباق | دانشمندان حفاظت | حسابرسان انرژی | مهندسان انرژی، به استثنای بادی و خورشیدی | اقتصاددانان محیط زیست | مهندسان محیط زیست | برنامه‌ریزان احیای محیط زیست | معلمان علوم محیط زیست، پس از متوسطه | دانشمندان و متخصصان محیط زیست، از جمله بهداشت | اکولوژیست‌های صنعتی | مدیران پروژه فناوری اطلاعات | تحلیل‌گران مدیریت | متخصصان مدیریت پروژه | متخصصان پایداری | برنامه‌ریزان شهری و منطقه‌ای | متخصصان منابع آب | مدیران توسعه انرژی بادی</t>
+          <t>متخصصان بازآفرینی زمین‌های قهوه‌ای و مدیران سایت | مدیران ارشد اجرایی | تحلیل‌گران سیاست تغییرات اقلیمی | مدیران انطباق | دانشمندان حفاظت | بازرسان انرژی | مهندسان انرژی، به جز باد و خورشید | اقتصاددانان محیط‌زیست | مهندسان محیط زیست | برنامه‌ریزان احیای محیط‌زیست | مدرسان علوم محیطی، پس از متوسطه | دانشمندان و متخصصان محیط زیست، شامل بهداشت | بوم‌شناسان صنعتی | مدیران پروژه فناوری اطلاعات | تحلیل‌گران مدیریت | متخصصان مدیریت پروژه | متخصصان پایداری | برنامه‌ریزان شهری و منطقه‌ای | متخصصان منابع آب | مدیران توسعه انرژی بادی</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -617,32 +617,32 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ADP Workforce Now | AMG Teleran SalesInSync | Act! | ActionWare | Adobe Acrobat | نرم‌افزار Adobe Creative Cloud | Adobe Photoshop | Airtable | نرم‌افزار Amazon Web Services AWS | Apache Hadoop | Apple Final Cut Pro | Apple Keynote | Apple macOS | Atlassian Confluence | Atlassian JIRA | Autodesk AutoCAD | Avidian Technologies Prophet | Blackbaud The Raiser's Edge | نرم‌افزار Blackboard | CNC Mastercam | نرم‌افزار رایانش ابری Citrix | سیستم کنترل اطلاعات مشتری CICS | نرم‌افزار پایگاه داده | Datawatch Monarch | Deacom ERP | Delphi Technology | Dropbox | Dynamic Energy Systems MedAct | Eko | Evernote | زبان نشانه‌گذاری توسعه‌پذیر XML | Facebook | FileMaker Pro | Flipgrid | نرم‌افزار حسابداری صندوق | نرم‌افزار سیستم اطلاعات جغرافیایی GIS | Google Ads | Google Analytics | Google Docs | Google Drive | Google Slides | GroupMe | HEAT Software GoldMine | نرم‌افزار HubSpot | نرم‌افزار مدیریت منابع انسانی HRMS | IBM Cognos Impromptu | IBM Domino | IBM InfoSphere DataStage | IBM Notes | نرم‌افزار IBM Power Systems | IBM SPSS Statistics | InnQuest Software roomMaster | Intuit QuickBooks | زبان کنترل کار JCL | Kronos Workforce Payroll | Kronos Workforce Timekeeper | LSA Visual Easy Lean | LexisNexis | LinkedIn | Marketo Marketing Automation | Maximizer Software Maximizer Enterprise | McAfee | نرم‌افزار کدگذاری شرایط پزشکی | MicroStrategy | Microsoft Access | Microsoft Dynamics | Microsoft Dynamics GP | Microsoft Excel | Microsoft Exchange | Microsoft FrontPage | Microsoft Internet Explorer | نرم‌افزار Microsoft Office | Microsoft OneNote | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SQL Server | Microsoft SharePoint | Microsoft Visio | Microsoft Visual Basic | Microsoft Visual Basic for Applications VBA | Microsoft Windows | Microsoft Word | Minitab | Mozilla Firefox | Mozilla Thunderbird | Nagios | NetSuite ERP | NetSuite NetCRM | نرم‌افزار امنیت سایبری NortonLifeLock | Oracle Business Intelligence Enterprise Edition | Oracle Database | Oracle E-Business Suite Financials | Oracle Eloqua | Oracle Fusion Applications | Oracle Hyperion | Oracle JD Edwards EnterpriseOne | Oracle PeopleSoft | Oracle PeopleSoft Financials | Oracle Primavera Enterprise Project Portfolio Management | Oracle Solaris | Oracle Taleo | نرم‌افزار حقوق و دستمزد | نرم‌افزار زمان‌بندی پرسنل | PostgreSQL | Puppet | Qlik Tech QlikView | Quest Erwin Data Modeler | R | Realization Streamliner | SAP Business Objects | SAP Crystal Reports | نرم‌افزار SAP | SAS | Sage 50 Accounting | Sage MAS 500 | نرم‌افزار Salesforce | Salesforce.com Salesforce CRM | Savant MobileRanger | Screencastify | SeaMonkey | اسکریپت Shell | Siemens NX | Slack | سایت‌های رسانه‌های اجتماعی | Software on Sailboats Desktop Sales Manager | Splunk Enterprise | StataCorp Stata | زبان پرس و جوی ساختاریافته SQL | Sugar CRM | نرم‌افزار کنترل نظارتی و اکتساب داده SCADA | Tableau | نرم‌افزار مالیات | Teradata Database | The MathWorks MATLAB | Vanguard Software Vanguard Sales Manager | Veritas NetBackup | نرم‌افزار Yardi | YouTube | vtiger CRM</t>
+          <t>ADP Workforce Now | AMG Teleran SalesInSync | Act! | ActionWare | Adobe Acrobat | نرم‌افزار Adobe Creative Cloud | Adobe Photoshop | Airtable | نرم‌افزار Amazon Web Services AWS | Apache Hadoop | Apple Final Cut Pro | Apple Keynote | Apple macOS | Atlassian Confluence | Atlassian JIRA | Autodesk AutoCAD | Avidian Technologies Prophet | Blackbaud The Raiser's Edge | نرم‌افزار Blackboard | CNC Mastercam | نرم‌افزار رایانش ابری Citrix | سیستم کنترل اطلاعات مشتری CICS | نرم‌افزار پایگاه داده | Datawatch Monarch | Deacom ERP | Delphi Technology | Dropbox | Dynamic Energy Systems MedAct | Eko | Evernote | زبان نشانه‌گذاری توسعه‌پذیر XML | Facebook | FileMaker Pro | Flipgrid | نرم‌افزار حسابداری صندوق | نرم‌افزار سیستم اطلاعات جغرافیایی GIS | Google Ads | Google Analytics | Google Docs | Google Drive | Google Slides | GroupMe | HEAT Software GoldMine | نرم‌افزار HubSpot | نرم‌افزار مدیریت منابع انسانی HRMS | IBM Cognos Impromptu | IBM Domino | IBM InfoSphere DataStage | IBM Notes | نرم‌افزار IBM Power Systems | IBM SPSS Statistics | InnQuest Software roomMaster | Intuit QuickBooks | زبان کنترل کار JCL | Kronos Workforce Payroll | Kronos Workforce Timekeeper | LSA Visual Easy Lean | LexisNexis | LinkedIn | Marketo Marketing Automation | Maximizer Software Maximizer Enterprise | McAfee | نرم‌افزار کدگذاری شرایط پزشکی | MicroStrategy | Microsoft Access | Microsoft Dynamics | Microsoft Dynamics GP | Microsoft Excel | Microsoft Exchange | Microsoft FrontPage | Microsoft Internet Explorer | نرم‌افزار Microsoft Office | Microsoft OneNote | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SQL Server | Microsoft SharePoint | Microsoft Visio | Microsoft Visual Basic | Microsoft Visual Basic for Applications VBA | Microsoft Windows | Microsoft Word | Minitab | Mozilla Firefox | Mozilla Thunderbird | Nagios | NetSuite ERP | NetSuite NetCRM | نرم‌افزار امنیت سایبری NortonLifeLock | Oracle Business Intelligence Enterprise Edition | Oracle Database | Oracle E-Business Suite Financials | Oracle Eloqua | Oracle Fusion Applications | Oracle Hyperion | Oracle JD Edwards EnterpriseOne | Oracle PeopleSoft | Oracle PeopleSoft Financials | Oracle Primavera Enterprise Project Portfolio Management | Oracle Solaris | Oracle Taleo | نرم‌افزار حقوق و دستمزد | نرم‌افزار زمان‌بندی پرسنل | PostgreSQL | Puppet | Qlik Tech QlikView | Quest Erwin Data Modeler | R | Realization Streamliner | SAP Business Objects | SAP Crystal Reports | نرم‌افزار SAP | SAS | Sage 50 Accounting | Sage MAS 500 | نرم‌افزار Salesforce | Salesforce.com Salesforce CRM | Savant MobileRanger | Screencastify | SeaMonkey | Shell script | Siemens NX | Slack | سایت‌های رسانه‌های اجتماعی | Software on Sailboats Desktop Sales Manager | Splunk Enterprise | StataCorp Stata | زبان پرس‌وجوی ساختاریافته SQL | Sugar CRM | نرم‌افزار کنترل نظارتی و گردآوری داده SCADA | Tableau | نرم‌افزار مالیاتی | Teradata Database | The MathWorks MATLAB | Vanguard Software Vanguard Sales Manager | Veritas NetBackup | نرم‌افزار Yardi | YouTube | vtiger CRM</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>نظارت | صحبت کردن | گوش دادن فعال | درک مطلب | تفکر انتقادی | یادگیری فعال | نوشتن | استراتژی‌های یادگیری</t>
+          <t>نظارت | سخن گفتن | گوش دادن فعال | درک مطلب | تفکر انتقادی | یادگیری فعال | نگارش | راهبردهای یادگیری</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>مدیریت و اداره | خدمات مشتری و شخصی | زبان انگلیسی | تولید و پردازش | ریاضیات | پرسنل و منابع انسانی | اداری | اقتصاد و حسابداری</t>
+          <t>مدیریت و اداره | خدمات مشتری و شخصی | زبان انگلیسی | تولید و فرآوری | ریاضیات | پرسنل و منابع انسانی | اداری | اقتصاد و حسابداری</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>بیان کتبی | درک شفاهی | درک کتبی | بیان شفاهی | حساسیت به مشکل | استدلال قیاسی | وضوح گفتار | تشخیص گفتار | بینایی نزدیک | مرتب‌سازی اطلاعات | استدلال استقرایی | انعطاف‌پذیری دسته‌بندی | روانی ایده‌ها | اصالت</t>
+          <t>بیان کتبی | درک شفاهی | درک کتبی | بیان شفاهی | حساسیت به مسئله | استدلال قیاسی | وضوح گفتار | تشخیص گفتار | بینایی نزدیک | ترتیب‌دهی اطلاعات | استدلال استقرایی | انعطاف‌پذیری دسته‌بندی | روانی ایده‌ها | اصالت</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>فرکانس تصمیم‌گیری | ایمیل | بحث‌های چهره به چهره با افراد و درون تیم‌ها | آزادی در تصمیم‌گیری | مکالمات تلفنی | تعیین وظایف، اولویت‌ها و اهداف | تماس با دیگران | کار با یا مشارکت در یک گروه کاری یا تیم | بهداشت و ایمنی سایر کارگران | تأثیر تصمیمات بر همکاران یا نتایج شرکت | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | فضای داخلی، با محیط کنترل‌شده | پیامدهای کاری و نتایج سایر کارگران | اهمیت دقیق یا صحیح بودن | فشار زمانی | نامه‌ها و یادداشت‌های کتبی</t>
+          <t>فراوانی تصمیم‌گیری | ایمیل | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | آزادی در تصمیم‌گیری | مکالمات تلفنی | تعیین وظایف، اولویت‌ها و اهداف | ارتباط با دیگران | کار با یا مشارکت در یک گروه کاری یا تیم | سلامت و ایمنی سایر کارکنان | تأثیر تصمیمات بر همکاران یا نتایج شرکت | تعامل با مشتریان خارجی یا عموم مردم | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | محیط داخلی، دارای کنترل شرایط محیطی | پیامدهای کاری و نتایج سایر کارکنان | اهمیت دقیق یا درست بودن | فشار زمانی | نامه‌ها و یادداشت‌های کتبی</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>مدیران خدمات اداری | مدیران ارشد اجرایی | مدیران ساخت و ساز | مدیران تسهیلات | سرپرستان خط اول کارگران مشاغل ساختمانی و استخراج | سرپرستان خط اول کارگران سرگرمی و تفریح، به استثنای خدمات قمار | سرپرستان خط اول دستیاران، کارگران، و جابجاکنندگان مواد، دستی | سرپرستان خط اول کارگران خانه‌داری و نظافت | سرپرستان خط اول اپراتورهای ماشین‌آلات جابجایی مواد و وسایل نقلیه | سرپرستان خط اول مکانیک‌ها، نصاب‌ها، و تعمیرکاران | سرپرستان خط اول کارگران فروش غیر خرده‌فروشی | سرپرستان خط اول کارگران پشتیبانی اداری و دفتری | سرپرستان خط اول کارگران تولید و عملیات | مهندسان صنایع | مدیران تولید صنعتی | مدیران پروژه فناوری اطلاعات | تحلیل‌گران مدیریت | متخصصان مدیریت پروژه | مدیران فروش | مدیران حمل و نقل، ذخیره‌سازی، و توزیع</t>
+          <t>مدیران خدمات اداری | مدیران ارشد اجرایی | مدیران ساخت‌وساز | مدیران تسهیلات | سرپرستان خط اول مشاغل ساختمانی و کارگران استخراج | سرپرستان خط اول کارگران سرگرمی و تفریح، به جز خدمات قمار | سرپرستان خط اول کمک‌یارها، کارگران ساده و جابجا‌کنندگان دستی مواد | سرپرستان خط اول کارگران خانه‌داری و سرایداری | سرپرستان خط اول اپراتورهای ماشین‌آلات و وسایل نقلیه جابجایی مواد | سرپرستان خط اول مکانیک‌ها، نصابان و تعمیرکاران | سرپرستان رده اول کارکنان فروش غیرخرده‌فروشی | سرپرستان خط اول کارکنان دفتری و پشتیبانی اداری | سرپرستان رده اول کارگران تولید و بهره‌برداری | مهندسان صنایع | مدیران تولید صنعتی | مدیران پروژه فناوری اطلاعات | تحلیل‌گران مدیریت | متخصصان مدیریت پروژه | مدیران فروش | مدیران حمل‌ونقل، انبارداری و توزیع</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -674,32 +674,32 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Adobe Acrobat | Adobe FrameMaker | Antenna House | Apple Numbers for Mac | Apple iWork Keynote | Apple iWork Pages | Cisco AnyConnect | Cisco Webex | Corel WordPerfect Office Suite | GoodReader | IBM Domino | Legislative Automative Workflow System LAWS | LogMeIn GoToMeeting | نرم‌افزار نقشه‌برداری | نرم‌افزار زمان‌بندی جلسه | Microsoft Access | Microsoft Excel | Microsoft Exchange | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft SQL Server | Microsoft SharePoint | Microsoft Visual Basic | Microsoft Word | PTC Arbortext | Penultimate | Rocket/Folio NXT | زبان پرس و جوی ساختاریافته SQL | نرم‌افزار مرورگر وب | Windows Media Player | XMetaL Author | iAnnotate</t>
+          <t>Adobe Acrobat | Adobe FrameMaker | Antenna House | Apple Numbers for Mac | Apple iWork Keynote | Apple iWork Pages | Cisco AnyConnect | Cisco Webex | Corel WordPerfect Office Suite | GoodReader | IBM Domino | Legislative Automative Workflow System LAWS | LogMeIn GoToMeeting | نرم‌افزار نقشه‌برداری | نرم‌افزار زمان‌بندی جلسه | Microsoft Access | Microsoft Excel | Microsoft Exchange | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft SQL Server | Microsoft SharePoint | Microsoft Visual Basic | Microsoft Word | PTC Arbortext | Penultimate | Rocket/Folio NXT | زبان پرس‌وجوی ساختاریافته SQL | نرم‌افزار مرورگر وب | Windows Media Player | XMetaL Author | iAnnotate</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>درک مطلب | تفکر انتقادی | گوش دادن فعال | صحبت کردن | نوشتن | نظارت | یادگیری فعال | استراتژی‌های یادگیری</t>
+          <t>درک مطلب | تفکر انتقادی | گوش دادن فعال | سخن گفتن | نگارش | نظارت | یادگیری فعال | راهبردهای یادگیری</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>قانون و دولت | زبان انگلیسی | مدیریت و اداره | ارتباطات و رسانه | اقتصاد و حسابداری | جامعه‌شناسی و انسان‌شناسی | ایمنی و امنیت عمومی | پرسنل و منابع انسانی | تاریخ و باستان‌شناسی | روانشناسی</t>
+          <t>قانون و دولت | زبان انگلیسی | مدیریت و اداره | ارتباطات و رسانه | اقتصاد و حسابداری | جامعه‌شناسی و انسان‌شناسی | ایمنی و امنیت عمومی | پرسنل و منابع انسانی | تاریخ و باستان‌شناسی | روان‌شناسی</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | استدلال قیاسی | استدلال استقرایی | مرتب‌سازی اطلاعات | حساسیت به مشکل | بینایی نزدیک | وضوح گفتار | تشخیص گفتار | انعطاف‌پذیری دسته‌بندی | روانی ایده‌ها | اصالت | توجه انتخابی | اشتراک زمانی | تجسم | حفظ کردن</t>
+          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | استدلال قیاسی | استدلال استقرایی | ترتیب‌دهی اطلاعات | حساسیت به مسئله | بینایی نزدیک | وضوح گفتار | تشخیص گفتار | انعطاف‌پذیری دسته‌بندی | روانی ایده‌ها | اصالت | توجه انتخابی | تقسیم توجه | تجسم | حفظ کردن</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>ایمیل | مکالمات تلفنی | بحث‌های چهره به چهره با افراد و درون تیم‌ها | فضای داخلی، با محیط کنترل‌شده | صرف زمان برای نشستن | تماس با دیگران | کار با یا مشارکت در یک گروه کاری یا تیم | آزادی در تصمیم‌گیری | تعیین وظایف، اولویت‌ها و اهداف | اهمیت دقیق یا صحیح بودن | فشار زمانی | نامه‌ها و یادداشت‌های کتبی | فرکانس تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | پیامدهای کاری و نتایج سایر کارگران | سخنرانی عمومی | موقعیت‌های تعارض | سطح رقابت</t>
+          <t>ایمیل | مکالمات تلفنی | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | محیط داخلی، دارای کنترل شرایط محیطی | صرف زمان برای نشستن | ارتباط با دیگران | کار با یا مشارکت در یک گروه کاری یا تیم | آزادی در تصمیم‌گیری | تعیین وظایف، اولویت‌ها و اهداف | اهمیت دقیق یا درست بودن | فشار زمانی | نامه‌ها و یادداشت‌های کتبی | فراوانی تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | تعامل با مشتریان خارجی یا عموم مردم | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | پیامدهای کاری و نتایج سایر کارکنان | سخنرانی عمومی | موقعیت‌های تعارض | سطح رقابت</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>قضات حقوق اداری، داوران، و افسران استماع | داوران، میانجی‌گران، و سازش‌دهندگان | مدیران ارشد اجرایی | کارمندان دادگاه، شهرداری، و مجوز | مدیران، فعالیت‌های مذهبی و آموزش | مدیران آموزش، مهدکودک تا متوسطه | مدیران آموزش، پس از متوسطه | نمایندگان و افسران فرصت برابر | منشی‌های اجرایی و دستیاران اداری اجرایی | مدیران عمومی و عملیات | کارمندان حقوقی قضایی | متخصصان روابط کار | وکلا | نمایندگان بیمار | معلمان علوم سیاسی، پس از متوسطه | دانشمندان علوم سیاسی | متخصصان روابط عمومی | مدیران خدمات اجتماعی و جامعه | دستیاران خدمات اجتماعی و انسانی | خزانه‌داران و کنترل‌کننده‌ها</t>
+          <t>قضات حقوق اداری، داوران و مسئولان رسیدگی | داوران، میانجی‌گران و مصالحه‌گران | مدیران ارشد اجرایی | کارمندان دادگاه، شهرداری و مجوز | مدیران، فعالیت‌ها و آموزش‌های مذهبی | مدیران آموزشی، مهدکودک تا دبیرستان | مدیران آموزشی، پس از متوسطه | نمایندگان و افسران فرصت‌های برابر | منشی‌های اجرایی و دستیاران اداری اجرایی | مدیران عمومی و عملیات | کارمندان حقوقی قضایی | متخصصان روابط کار | وکلا | نمایندگان بیمار | استادان علوم سیاسی، پس از متوسطه | دانشمندان علوم سیاسی | متخصصان روابط عمومی | مدیران خدمات اجتماعی و جامعه | دستیاران خدمات اجتماعی و انسانی | خزانه‌داران و کنترل‌کنندگان</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -731,32 +731,32 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Actuate BIRT | AdRelevance | Adobe Acrobat | Adobe Acrobat Reader | Adobe After Effects | نرم‌افزار Adobe Creative Cloud | Adobe Dreamweaver | Adobe Experience Manager (AEM) | Adobe Illustrator | Adobe InDesign | Adobe PageMaker | Adobe Photoshop | Adobe Premiere Pro | Apple Final Cut Pro | Apple iMovie | Avid Media Composer | Brainworks | نرم‌افزار تحلیل کسب‌وکار | Constant Contact | نرم‌افزار تجسم داده | نرم‌افزار انبار داده | نرم‌افزار پایگاه داده | Drupal | نرم‌افزار ایمیل | Experience in Software Webplanner | زبان نشانه‌گذاری توسعه‌پذیر XML | Facebook | Google Ads | Google Analytics | Google DoubleClick | Hootsuite | نرم‌افزار HubSpot | زبان نشانه‌گذاری ابرمتن HTML | IBM Lotus Notes | Instagram | نرم‌افزار ردیابی موجودی | JavaScript | LinkedIn | MailChimp | MarketSharp | Marketo Marketing Automation | Microsoft Access | Microsoft Dynamics | Microsoft Dynamics Marketing | Microsoft Excel | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SQL Server | Microsoft SharePoint | Microsoft Windows | Microsoft Word | Oracle Eloqua | PaloAlto Advertising Plan Pro | Pinterest | نرم‌افزار انتشار سازمانی Quark | Relex Weibull | نرم‌افزار SAP | نرم‌افزار Salesforce | نرم‌افزار زمان‌بندی | نرم‌افزار رسانه‌های اجتماعی | زبان پرس و جوی ساختاریافته SQL | Tableau | Twitter | Vimeo | نرم‌افزار مرورگر وب | WebTrends Analytics | نرم‌افزار Webtrends | WordPress | YouTube</t>
+          <t>Actuate BIRT | AdRelevance | Adobe Acrobat | Adobe Acrobat Reader | Adobe After Effects | نرم‌افزار Adobe Creative Cloud | Adobe Dreamweaver | Adobe Experience Manager (AEM) | Adobe Illustrator | Adobe InDesign | Adobe PageMaker | Adobe Photoshop | Adobe Premiere Pro | Apple Final Cut Pro | Apple iMovie | Avid Media Composer | Brainworks | نرم‌افزار تحلیل کسب‌وکار | Constant Contact | نرم‌افزار تجسم داده | نرم‌افزار انبار داده | نرم‌افزار پایگاه داده | Drupal | نرم‌افزار ایمیل | Experience in Software Webplanner | زبان نشانه‌گذاری توسعه‌پذیر XML | Facebook | Google Ads | Google Analytics | Google DoubleClick | Hootsuite | نرم‌افزار HubSpot | زبان نشانه‌گذاری ابرمتن HTML | IBM Lotus Notes | Instagram | نرم‌افزار ردیابی موجودی | JavaScript | LinkedIn | MailChimp | MarketSharp | Marketo Marketing Automation | Microsoft Access | Microsoft Dynamics | Microsoft Dynamics Marketing | Microsoft Excel | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SQL Server | Microsoft SharePoint | Microsoft Windows | Microsoft Word | Oracle Eloqua | PaloAlto Advertising Plan Pro | Pinterest | نرم‌افزار نشر سازمانی Quark | Relex Weibull | نرم‌افزار SAP | نرم‌افزار Salesforce | نرم‌افزار زمان‌بندی | نرم‌افزار رسانه‌های اجتماعی | زبان پرس‌وجوی ساختاریافته SQL | Tableau | Twitter | Vimeo | نرم‌افزار مرورگر وب | WebTrends Analytics | نرم‌افزار Webtrends | WordPress | YouTube</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>گوش دادن فعال | تفکر انتقادی | صحبت کردن | نوشتن | درک مطلب | نظارت | یادگیری فعال | استراتژی‌های یادگیری | ریاضیات</t>
+          <t>گوش دادن فعال | تفکر انتقادی | سخن گفتن | نگارش | درک مطلب | نظارت | یادگیری فعال | راهبردهای یادگیری | ریاضیات</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>فروش و بازاریابی | زبان انگلیسی | ارتباطات و رسانه | خدمات مشتری و شخصی | مدیریت و اداره | رایانه‌ها و الکترونیک | اداری | ریاضیات | اقتصاد و حسابداری</t>
+          <t>فروش و بازاریابی | زبان انگلیسی | ارتباطات و رسانه | خدمات مشتری و شخصی | مدیریت و اداره | رایانه و الکترونیک | اداری | ریاضیات | اقتصاد و حسابداری</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>بیان شفاهی | درک شفاهی | درک کتبی | وضوح گفتار | بیان کتبی | استدلال قیاسی | تشخیص گفتار | بینایی نزدیک | روانی ایده‌ها | اصالت | حساسیت به مشکل | استدلال استقرایی | انعطاف‌پذیری دسته‌بندی | تجسم | مرتب‌سازی اطلاعات | انعطاف‌پذیری انسداد | استدلال ریاضی</t>
+          <t>بیان شفاهی | درک شفاهی | درک کتبی | وضوح گفتار | بیان کتبی | استدلال قیاسی | تشخیص گفتار | بینایی نزدیک | روانی ایده‌ها | اصالت | حساسیت به مسئله | استدلال استقرایی | انعطاف‌پذیری دسته‌بندی | تجسم | ترتیب‌دهی اطلاعات | انعطاف‌پذیری بستار | استدلال ریاضی</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>ایمیل | بحث‌های چهره به چهره با افراد و درون تیم‌ها | مکالمات تلفنی | تماس با دیگران | فضای داخلی، با محیط کنترل‌شده | کار با یا مشارکت در یک گروه کاری یا تیم | فشار زمانی | صرف زمان برای نشستن | فرکانس تصمیم‌گیری | اهمیت دقیق یا صحیح بودن | تعیین وظایف، اولویت‌ها و اهداف | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | آزادی در تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | پیامدهای کاری و نتایج سایر کارگران | نامه‌ها و یادداشت‌های کتبی</t>
+          <t>ایمیل | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | مکالمات تلفنی | ارتباط با دیگران | محیط داخلی، دارای کنترل شرایط محیطی | کار با یا مشارکت در یک گروه کاری یا تیم | فشار زمانی | صرف زمان برای نشستن | فراوانی تصمیم‌گیری | اهمیت دقیق یا درست بودن | تعیین وظایف، اولویت‌ها و اهداف | تعامل با مشتریان خارجی یا عموم مردم | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | آزادی در تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | پیامدهای کاری و نتایج سایر کارکنان | نامه‌ها و یادداشت‌های کتبی</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>نمایندگان فروش تبلیغات | نمایندگان و مدیران کسب‌وکار هنرمندان، مجریان، و ورزشکاران | مدیران هنری | تحلیل‌گران هوش تجاری | جمع‌آوری‌کنندگان کمک‌های مالی | مدیران جمع‌آوری کمک‌های مالی | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | مدیران بازاریابی | نمایش‌دهندگان کالا و تزئین‌کنندگان ویترین | بازرگانان آنلاین | مدیران روابط عمومی | متخصصان روابط عمومی | مدیران خرید | مدیران فروش | نمایندگان فروش خدمات، به استثنای تبلیغات، بیمه، خدمات مالی، و سفر | استراتژیست‌های بازاریابی جستجو | بازاریابان تلفنی | مدیران وب | نویسندگان و مؤلفان</t>
+          <t>نمایندگان فروش تبلیغات | نمایندگان و مدیران تجاری هنرمندان، اجراکنندگان و ورزشکاران | مدیران هنری | تحلیلگران هوش تجاری | جمع‌آوری‌کنندگان کمک مالی | مدیران جمع‌آوری کمک‌های مالی | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | مدیران بازاریابی | چیدمان‌کنندگان کالا و تزئین‌کنندگان ویترین | تاجران آنلاین | مدیران روابط عمومی | متخصصان روابط عمومی | مدیران خرید | مدیران فروش | نمایندگان فروش خدمات، به جز تبلیغات، بیمه، خدمات مالی و سفر | استراتژیست‌های بازاریابی جستجو | بازاریابان تلفنی | مدیران وب | نویسندگان و مؤلفان</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -788,32 +788,32 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>AEC Software FastTrack Schedule | AdSense Tracker | Adobe Acrobat | Adobe Acrobat Reader | Adobe ActionScript | Adobe After Effects | نرم‌افزار Adobe Creative Cloud | Adobe Dreamweaver | Adobe Illustrator | Adobe InDesign | Adobe Photoshop | Airtable | Amazon Redshift | نرم‌افزار Amazon Web Services AWS | Apache Cassandra | Apache Hadoop | Apache Hive | Apache Pig | Apache Solr | Apple Final Cut Pro | Apple Keynote | Apple macOS | Armand Morin MultiTrack Generator | Asana | Atlassian Confluence | Atlassian JIRA | Blackbaud The Raiser's Edge | C | Canva | برگه‌های سبک آبشاری CSS | نرم‌افزار رایانش ابری Citrix | ClearEDGE | Constant Contact | نرم‌افزار گزارش‌گیری پایگاه داده | نرم‌افزار پایگاه داده | Databox | Delphi Technology | Dropbox | Drupal | زبان نشانه‌گذاری ابرمتن پویا DHTML | Eko | Elasticsearch | Evernote | زبان نشانه‌گذاری ابرمتن توسعه‌پذیر XHTML | زبان نشانه‌گذاری توسعه‌پذیر XML | Facebook | Figma | FileMaker Pro | Flipgrid | نرم‌افزار حسابداری صندوق | GitHub | Google Ads | Google Analytics | Google Docs | Google Drive | Google Looker Analytics | Google Meet | Google Slides | نرم‌افزار HubSpot | زبان نشانه‌گذاری ابرمتن HTML | IBM Cognos Impromptu | IBM Domino | IBM InfoSphere DataStage | IBM Notes | نرم‌افزار IBM Power Systems | IBM SPSS Statistics | Instagram | Intuit QuickBooks | JamBoard | JavaScript | Jupyter Notebook | Kapwing | LAMP Stack | LexisNexis | LinkedIn | LogMeIn GoToMeeting | LogMeIn GoToWebinar | Lyris HQ Web-Analytics Solution | MarketSharp | Marketo Marketing Automation | McAfee | Mentimeter | MicroStrategy | Microsoft Access | نرم‌افزار Microsoft Azure | Microsoft Dynamics | Microsoft Excel | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SQL Server | Microsoft SharePoint | Microsoft Teams | Microsoft Visio | Microsoft Visual Basic | Microsoft Visual Basic Scripting Edition VBScript | Microsoft Visual Basic for Applications VBA | Microsoft Word | Minitab | MySQL | Nearpod | Nedstat Sitestat | NetSuite ERP | NoSQL | نرم‌افزار امنیت سایبری NortonLifeLock | نرم‌افزار گزارش‌گیری تبلیغات آنلاین | Oracle Beehive | Oracle Business Intelligence Enterprise Edition | Oracle Database | Oracle E-Business Suite Financials | Oracle Eloqua | Oracle Fusion Applications | Oracle Hyperion | Oracle JavaServer Pages JSP | Oracle PL/SQL | Oracle PeopleSoft | Oracle PeopleSoft Financials | Oracle Siebel Server Sync | PHP | Padlet | Python | QAD Marketing Automation | Qlik Tech QlikView | R | Ruby | Ruby on Rails | SAP Business Objects | نرم‌افزار SAP | SAS | Sage SalesLogix | نرم‌افزار Salesforce | Salesforce.com Salesforce CRM | Screencast-O-Matic | Screencastify | Slack | SmugMug Flickr | سایت‌های رسانه‌های اجتماعی | نرم‌افزار به عنوان سرویس SaaS | Splunk Enterprise | StataCorp Stata | زبان پرس و جوی ساختاریافته SQL | Swift | Tableau | نرم‌افزار مالیات | Teradata Database | The MathWorks MATLAB | TikTok | WeVideo | نرم‌افزار مرورگر وب | WordPress | نرم‌افزار Yardi | YouTube</t>
+          <t>AEC Software FastTrack Schedule | AdSense Tracker | Adobe Acrobat | Adobe Acrobat Reader | Adobe ActionScript | Adobe After Effects | نرم‌افزار Adobe Creative Cloud | Adobe Dreamweaver | Adobe Illustrator | Adobe InDesign | Adobe Photoshop | Airtable | Amazon Redshift | نرم‌افزار Amazon Web Services AWS | Apache Cassandra | Apache Hadoop | Apache Hive | Apache Pig | Apache Solr | Apple Final Cut Pro | Apple Keynote | Apple macOS | Armand Morin MultiTrack Generator | Asana | Atlassian Confluence | Atlassian JIRA | Blackbaud The Raiser's Edge | C | Canva | برگه‌های سبک آبشاری CSS | نرم‌افزار رایانش ابری Citrix | ClearEDGE | Constant Contact | نرم‌افزار گزارش‌گیری پایگاه داده | نرم‌افزار پایگاه داده | Databox | Delphi Technology | Dropbox | Drupal | زبان نشانه‌گذاری ابرمتن پویا DHTML | Eko | Elasticsearch | Evernote | زبان نشانه‌گذاری ابرمتن توسعه‌پذیر XHTML | زبان نشانه‌گذاری توسعه‌پذیر XML | Facebook | Figma | FileMaker Pro | Flipgrid | نرم‌افزار حسابداری صندوق | GitHub | Google Ads | Google Analytics | Google Docs | Google Drive | Google Looker Analytics | Google Meet | Google Slides | نرم‌افزار HubSpot | زبان نشانه‌گذاری ابرمتن HTML | IBM Cognos Impromptu | IBM Domino | IBM InfoSphere DataStage | IBM Notes | نرم‌افزار IBM Power Systems | IBM SPSS Statistics | Instagram | Intuit QuickBooks | JamBoard | JavaScript | Jupyter Notebook | Kapwing | LAMP Stack | LexisNexis | LinkedIn | LogMeIn GoToMeeting | LogMeIn GoToWebinar | Lyris HQ Web-Analytics Solution | MarketSharp | Marketo Marketing Automation | McAfee | Mentimeter | MicroStrategy | Microsoft Access | نرم‌افزار Microsoft Azure | Microsoft Dynamics | Microsoft Excel | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SQL Server | Microsoft SharePoint | Microsoft Teams | Microsoft Visio | Microsoft Visual Basic | Microsoft Visual Basic Scripting Edition VBScript | Microsoft Visual Basic for Applications VBA | Microsoft Word | Minitab | MySQL | Nearpod | Nedstat Sitestat | NetSuite ERP | NoSQL | نرم‌افزار امنیت سایبری NortonLifeLock | نرم‌افزار گزارش‌گیری تبلیغات آنلاین | Oracle Beehive | Oracle Business Intelligence Enterprise Edition | Oracle Database | Oracle E-Business Suite Financials | Oracle Eloqua | Oracle Fusion Applications | Oracle Hyperion | Oracle JavaServer Pages JSP | Oracle PL/SQL | Oracle PeopleSoft | Oracle PeopleSoft Financials | Oracle Siebel Server Sync | PHP | Padlet | Python | QAD Marketing Automation | Qlik Tech QlikView | R | Ruby | Ruby on Rails | SAP Business Objects | نرم‌افزار SAP | SAS | Sage SalesLogix | نرم‌افزار Salesforce | Salesforce.com Salesforce CRM | Screencast-O-Matic | Screencastify | Slack | SmugMug Flickr | سایت‌های رسانه‌های اجتماعی | نرم‌افزار به عنوان سرویس SaaS | Splunk Enterprise | StataCorp Stata | زبان پرس‌وجوی ساختاریافته SQL | Swift | Tableau | نرم‌افزار مالیاتی | Teradata Database | The MathWorks MATLAB | TikTok | WeVideo | نرم‌افزار مرورگر وب | WordPress | نرم‌افزار Yardi | YouTube</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>درک مطلب | گوش دادن فعال | صحبت کردن | تفکر انتقادی | یادگیری فعال | نظارت | نوشتن | استراتژی‌های یادگیری</t>
+          <t>درک مطلب | گوش دادن فعال | سخن گفتن | تفکر انتقادی | یادگیری فعال | نظارت | نگارش | راهبردهای یادگیری</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>فروش و بازاریابی | زبان انگلیسی | مدیریت و اداره | خدمات مشتری و شخصی | ارتباطات و رسانه | رایانه‌ها و الکترونیک | ریاضیات | طراحی | اقتصاد و حسابداری | آموزش و تعلیم | اداری</t>
+          <t>فروش و بازاریابی | زبان انگلیسی | مدیریت و اداره | خدمات مشتری و شخصی | ارتباطات و رسانه | رایانه و الکترونیک | ریاضیات | طراحی | اقتصاد و حسابداری | آموزش و پرورش | اداری</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | استدلال قیاسی | استدلال استقرایی | روانی ایده‌ها | وضوح گفتار | اصالت | حساسیت به مشکل | تشخیص گفتار | بینایی نزدیک | مرتب‌سازی اطلاعات | انعطاف‌پذیری دسته‌بندی | سهولت در اعداد | استدلال ریاضی | تجسم | انعطاف‌پذیری انسداد</t>
+          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | استدلال قیاسی | استدلال استقرایی | روانی ایده‌ها | وضوح گفتار | اصالت | حساسیت به مسئله | تشخیص گفتار | بینایی نزدیک | ترتیب‌دهی اطلاعات | انعطاف‌پذیری دسته‌بندی | توانایی عددی | استدلال ریاضی | تجسم | انعطاف‌پذیری بستار</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>ایمیل | مکالمات تلفنی | بحث‌های چهره به چهره با افراد و درون تیم‌ها | کار با یا مشارکت در یک گروه کاری یا تیم | تعیین وظایف، اولویت‌ها و اهداف | تماس با دیگران | فضای داخلی، با محیط کنترل‌شده | آزادی در تصمیم‌گیری | صرف زمان برای نشستن | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | فشار زمانی | تأثیر تصمیمات بر همکاران یا نتایج شرکت | فرکانس تصمیم‌گیری | پیامدهای کاری و نتایج سایر کارگران | سطح رقابت | اهمیت دقیق یا صحیح بودن | نامه‌ها و یادداشت‌های کتبی</t>
+          <t>ایمیل | مکالمات تلفنی | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | کار با یا مشارکت در یک گروه کاری یا تیم | تعیین وظایف، اولویت‌ها و اهداف | ارتباط با دیگران | محیط داخلی، دارای کنترل شرایط محیطی | آزادی در تصمیم‌گیری | صرف زمان برای نشستن | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | تعامل با مشتریان خارجی یا عموم مردم | فشار زمانی | تأثیر تصمیمات بر همکاران یا نتایج شرکت | فراوانی تصمیم‌گیری | پیامدهای کاری و نتایج سایر کارکنان | سطح رقابت | اهمیت دقیق یا درست بودن | نامه‌ها و یادداشت‌های کتبی</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>نمایندگان فروش تبلیغات | مدیران تبلیغات و ترویج | تحلیل‌گران هوش تجاری | تحلیل‌گران مالی و سرمایه‌گذاری | مدیران عمومی و عملیات | مدیران پروژه فناوری اطلاعات | لجستیک‌دانان | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | بازرگانان آنلاین | متخصصان مدیریت پروژه | مدیران روابط عمومی | متخصصان روابط عمومی | مدیران خرید | مدیران فروش | نمایندگان فروش خدمات، به استثنای تبلیغات، بیمه، خدمات مالی، و سفر | استراتژیست‌های بازاریابی جستجو | نمایندگان فروش اوراق بهادار، کالاها، و خدمات مالی | خریداران عمده‌فروشی و خرده‌فروشی، به استثنای محصولات کشاورزی | نویسندگان و مؤلفان</t>
+          <t>نمایندگان فروش تبلیغات | مدیران تبلیغات و ترویج | تحلیلگران هوش تجاری | تحلیلگران مالی و سرمایه‌گذاری | مدیران عمومی و عملیات | مدیران پروژه فناوری اطلاعات | لجستیسین‌ها | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | تاجران آنلاین | متخصصان مدیریت پروژه | مدیران روابط عمومی | متخصصان روابط عمومی | مدیران خرید | مدیران فروش | نمایندگان فروش خدمات، به جز تبلیغات، بیمه، خدمات مالی و سفر | استراتژیست‌های بازاریابی جستجو | نمایندگان فروش اوراق بهادار، کالاها و خدمات مالی | خریداران عمده‌فروشی و خرده‌فروشی، به جز محصولات کشاورزی | نویسندگان و مؤلفان</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -845,32 +845,32 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Act! | Adobe Acrobat | Adobe ActionScript | نرم‌افزار Adobe Creative Cloud | Airtable | Apple Keynote | Avidian Technologies Prophet | Bentley MicroStation | Blackbaud The Raiser's Edge | نرم‌افزار مدیریت تماس | نرم‌افزار پایگاه داده | Delphi Discovery | Delphi Technology | Dropbox | Eclipse IDE | Eden Sales Manager | Eko | Facebook | FileMaker Pro | نرم‌افزار سیستم اطلاعات جغرافیایی GIS | Google Ads | Google Analytics | Google Docs | Google Drive | Google Meet | Google Sites | Google Slides | HEAT Software GoldMine | نرم‌افزار HubSpot | نرم‌افزار مدیریت منابع انسانی HRMS | زبان نشانه‌گذاری ابرمتن HTML | IBM Cognos Impromptu | IBM Notes | نرم‌افزار IBM Power Systems | IBM SPSS Statistics | نرم‌افزار موجودی | LexisNexis | LinkedIn | LogMeIn GoToMeeting | Marketo Marketing Automation | Maximizer Software Maximizer Enterprise | McAfee | MicroStrategy | Microsoft Access | نرم‌افزار Microsoft Azure | Microsoft Dynamics | Microsoft Dynamics GP | Microsoft Excel | Microsoft Exchange | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SQL Server | Microsoft SharePoint | Microsoft Teams | Microsoft Visio | Microsoft Visual Basic | Microsoft Visual Basic for Applications VBA | Microsoft Windows | Microsoft Word | Minitab | NetSuite ERP | NetSuite NetCRM | نرم‌افزار امنیت سایبری NortonLifeLock | Oracle Business Intelligence Enterprise Edition | Oracle Database | Oracle E-Business Suite Financials | Oracle Eloqua | Oracle Fusion Applications | Oracle Hyperion | Oracle JD Edwards EnterpriseOne | Oracle PeopleSoft | Oracle PeopleSoft Financials | Oracle Primavera Enterprise Project Portfolio Management | Oracle Taleo | Poll Everywhere | Qlik Tech QlikView | R | SAP Business Objects | SAP BusinessObjects Crystal Reports | SAP Crystal Reports | نرم‌افزار SAP | SAS | Sage 50 Accounting | نرم‌افزار Salesforce | Salesforce.com Salesforce CRM | نرم‌افزار زمان‌بندی | SmugMug Flickr | سایت‌های رسانه‌های اجتماعی | Software on Sailboats Desktop Sales Manager | Splunk Enterprise | زبان پرس و جوی ساختاریافته SQL | Tableau | نرم‌افزار مالیات | Teradata Database | Vanguard Software Vanguard Sales Manager | نرم‌افزار مرورگر وب | نرم‌افزار مدیریت نیروی کار | نرم‌افزار Yardi | YouTube | Zoom</t>
+          <t>Act! | Adobe Acrobat | Adobe ActionScript | نرم‌افزار Adobe Creative Cloud | Airtable | Apple Keynote | Avidian Technologies Prophet | Bentley MicroStation | Blackbaud The Raiser's Edge | نرم‌افزار مدیریت تماس | نرم‌افزار پایگاه داده | Delphi Discovery | Delphi Technology | Dropbox | Eclipse IDE | Eden Sales Manager | Eko | Facebook | FileMaker Pro | نرم‌افزار سیستم اطلاعات جغرافیایی GIS | Google Ads | Google Analytics | Google Docs | Google Drive | Google Meet | Google Sites | Google Slides | HEAT Software GoldMine | نرم‌افزار HubSpot | نرم‌افزار مدیریت منابع انسانی HRMS | زبان نشانه‌گذاری ابرمتن HTML | IBM Cognos Impromptu | IBM Notes | نرم‌افزار IBM Power Systems | IBM SPSS Statistics | نرم‌افزار موجودی | LexisNexis | LinkedIn | LogMeIn GoToMeeting | Marketo Marketing Automation | Maximizer Software Maximizer Enterprise | McAfee | MicroStrategy | Microsoft Access | نرم‌افزار Microsoft Azure | Microsoft Dynamics | Microsoft Dynamics GP | Microsoft Excel | Microsoft Exchange | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SQL Server | Microsoft SharePoint | Microsoft Teams | Microsoft Visio | Microsoft Visual Basic | Microsoft Visual Basic for Applications VBA | Microsoft Windows | Microsoft Word | Minitab | NetSuite ERP | NetSuite NetCRM | نرم‌افزار امنیت سایبری NortonLifeLock | Oracle Business Intelligence Enterprise Edition | Oracle Database | Oracle E-Business Suite Financials | Oracle Eloqua | Oracle Fusion Applications | Oracle Hyperion | Oracle JD Edwards EnterpriseOne | Oracle PeopleSoft | Oracle PeopleSoft Financials | Oracle Primavera Enterprise Project Portfolio Management | Oracle Taleo | Poll Everywhere | Qlik Tech QlikView | R | SAP Business Objects | SAP BusinessObjects Crystal Reports | SAP Crystal Reports | نرم‌افزار SAP | SAS | Sage 50 Accounting | نرم‌افزار Salesforce | Salesforce.com Salesforce CRM | نرم‌افزار زمان‌بندی | SmugMug Flickr | سایت‌های رسانه‌های اجتماعی | Software on Sailboats Desktop Sales Manager | Splunk Enterprise | زبان پرس‌وجوی ساختاریافته SQL | Tableau | نرم‌افزار مالیاتی | Teradata Database | Vanguard Software Vanguard Sales Manager | نرم‌افزار مرورگر وب | نرم‌افزار مدیریت نیروی کار | نرم‌افزار Yardi | YouTube | Zoom</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>گوش دادن فعال | صحبت کردن | نظارت | درک مطلب | تفکر انتقادی | یادگیری فعال | نوشتن | استراتژی‌های یادگیری | ریاضیات</t>
+          <t>گوش دادن فعال | سخن گفتن | نظارت | درک مطلب | تفکر انتقادی | یادگیری فعال | نگارش | راهبردهای یادگیری | ریاضیات</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>فروش و بازاریابی | خدمات مشتری و شخصی | زبان انگلیسی | مدیریت و اداره | پرسنل و منابع انسانی | آموزش و تعلیم | رایانه‌ها و الکترونیک | ارتباطات و رسانه | اقتصاد و حسابداری</t>
+          <t>فروش و بازاریابی | خدمات مشتری و شخصی | زبان انگلیسی | مدیریت و اداره | پرسنل و منابع انسانی | آموزش و پرورش | رایانه و الکترونیک | ارتباطات و رسانه | اقتصاد و حسابداری</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | حساسیت به مشکل | استدلال قیاسی | استدلال استقرایی | روانی ایده‌ها | اصالت | تشخیص گفتار | وضوح گفتار | انعطاف‌پذیری دسته‌بندی | بینایی نزدیک | مرتب‌سازی اطلاعات</t>
+          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | حساسیت به مسئله | استدلال قیاسی | استدلال استقرایی | روانی ایده‌ها | اصالت | تشخیص گفتار | وضوح گفتار | انعطاف‌پذیری دسته‌بندی | بینایی نزدیک | ترتیب‌دهی اطلاعات</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>ایمیل | مکالمات تلفنی | تماس با دیگران | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | بحث‌های چهره به چهره با افراد و درون تیم‌ها | کار با یا مشارکت در یک گروه کاری یا تیم | فضای داخلی، با محیط کنترل‌شده | تعیین وظایف، اولویت‌ها و اهداف | سطح رقابت | آزادی در تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | صرف زمان برای نشستن | فرکانس تصمیم‌گیری | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | نامه‌ها و یادداشت‌های کتبی | فشار زمانی | پیامدهای کاری و نتایج سایر کارگران | در یک وسیله نقلیه محصور یا کار با تجهیزات محصور | موقعیت‌های تعارض</t>
+          <t>ایمیل | مکالمات تلفنی | ارتباط با دیگران | تعامل با مشتریان خارجی یا عموم مردم | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | کار با یا مشارکت در یک گروه کاری یا تیم | محیط داخلی، دارای کنترل شرایط محیطی | تعیین وظایف، اولویت‌ها و اهداف | سطح رقابت | آزادی در تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | صرف زمان برای نشستن | فراوانی تصمیم‌گیری | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | نامه‌ها و یادداشت‌های کتبی | فشار زمانی | پیامدهای کاری و نتایج سایر کارکنان | در یک وسیله نقلیه محصور یا کار با تجهیزات محصور | موقعیت‌های تعارض</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>نمایندگان فروش تبلیغات | مدیران تبلیغات و ترویج | کارمندان کارگزاری | مدیران ارشد اجرایی | نمایندگان خدمات مشتری | تحلیل‌گران مالی و سرمایه‌گذاری | سرپرستان خط اول کارگران فروش غیر خرده‌فروشی | سرپرستان خط اول کارگران پشتیبانی اداری و دفتری | سرپرستان خط اول کارگران فروش خرده‌فروشی | مدیران عمومی و عملیات | لجستیک‌دانان | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | مدیران بازاریابی | بازرگانان آنلاین | نمایندگان خرید، به استثنای عمده‌فروشی، خرده‌فروشی، و محصولات کشاورزی | مدیران خرید | نمایندگان فروش خدمات، به استثنای تبلیغات، بیمه، خدمات مالی، و سفر | نمایندگان فروش اوراق بهادار، کالاها، و خدمات مالی | خریداران عمده‌فروشی و خرده‌فروشی، به استثنای محصولات کشاورزی</t>
+          <t>نمایندگان فروش تبلیغات | مدیران تبلیغات و ترویج | کارمندان کارگزاری | مدیران ارشد اجرایی | نمایندگان خدمات مشتریان | تحلیلگران مالی و سرمایه‌گذاری | سرپرستان رده اول کارکنان فروش غیرخرده‌فروشی | سرپرستان خط اول کارکنان دفتری و پشتیبانی اداری | سرپرستان رده اول کارکنان فروش خرده‌فروشی | مدیران عمومی و عملیات | لجستیسین‌ها | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | مدیران بازاریابی | تاجران آنلاین | نمایندگان خرید، به جز عمده‌فروشی، خرده‌فروشی و محصولات کشاورزی | مدیران خرید | نمایندگان فروش خدمات، به جز تبلیغات، بیمه، خدمات مالی و سفر | نمایندگان فروش اوراق بهادار، کالاها و خدمات مالی | خریداران عمده‌فروشی و خرده‌فروشی، به جز محصولات کشاورزی</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -907,27 +907,27 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>درک مطلب | تفکر انتقادی | گوش دادن فعال | صحبت کردن | نوشتن | نظارت | یادگیری فعال | استراتژی‌های یادگیری</t>
+          <t>درک مطلب | تفکر انتقادی | گوش دادن فعال | سخن گفتن | نگارش | نظارت | یادگیری فعال | راهبردهای یادگیری</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ارتباطات و رسانه | زبان انگلیسی | خدمات مشتری و شخصی | فروش و بازاریابی | مدیریت و اداره | پرسنل و منابع انسانی | رایانه‌ها و الکترونیک | روانشناسی | آموزش و تعلیم | جامعه‌شناسی و انسان‌شناسی</t>
+          <t>ارتباطات و رسانه | زبان انگلیسی | خدمات مشتری و شخصی | فروش و بازاریابی | مدیریت و اداره | پرسنل و منابع انسانی | رایانه و الکترونیک | روان‌شناسی | آموزش و پرورش | جامعه‌شناسی و انسان‌شناسی</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | استدلال قیاسی | استدلال استقرایی | مرتب‌سازی اطلاعات | حساسیت به مشکل | بینایی نزدیک | وضوح گفتار | تشخیص گفتار | انعطاف‌پذیری دسته‌بندی | روانی ایده‌ها | اصالت | توجه انتخابی | اشتراک زمانی | تجسم | حفظ کردن</t>
+          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | استدلال قیاسی | استدلال استقرایی | ترتیب‌دهی اطلاعات | حساسیت به مسئله | بینایی نزدیک | وضوح گفتار | تشخیص گفتار | انعطاف‌پذیری دسته‌بندی | روانی ایده‌ها | اصالت | توجه انتخابی | تقسیم توجه | تجسم | حفظ کردن</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ایمیل | مکالمات تلفنی | بحث‌های چهره به چهره با افراد و درون تیم‌ها | فضای داخلی، با محیط کنترل‌شده | صرف زمان برای نشستن | تماس با دیگران | کار با یا مشارکت در یک گروه کاری یا تیم | آزادی در تصمیم‌گیری | تعیین وظایف، اولویت‌ها و اهداف | اهمیت دقیق یا صحیح بودن | فشار زمانی | نامه‌ها و یادداشت‌های کتبی | فرکانس تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | پیامدهای کاری و نتایج سایر کارگران | سخنرانی عمومی | موقعیت‌های تعارض | سطح رقابت</t>
+          <t>ایمیل | مکالمات تلفنی | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | محیط داخلی، دارای کنترل شرایط محیطی | صرف زمان برای نشستن | ارتباط با دیگران | کار با یا مشارکت در یک گروه کاری یا تیم | آزادی در تصمیم‌گیری | تعیین وظایف، اولویت‌ها و اهداف | اهمیت دقیق یا درست بودن | فشار زمانی | نامه‌ها و یادداشت‌های کتبی | فراوانی تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | تعامل با مشتریان خارجی یا عموم مردم | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | پیامدهای کاری و نتایج سایر کارکنان | سخنرانی عمومی | موقعیت‌های تعارض | سطح رقابت</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>مدیران خدمات اداری | نمایندگان فروش تبلیغات | مدیران تبلیغات و ترویج | تحلیل‌گران هوش تجاری | معلمان کسب‌وکار، پس از متوسطه | مدیران ارشد اجرایی | معلمان ارتباطات، پس از متوسطه | منشی‌های اجرایی و دستیاران اداری اجرایی | مدیران جمع‌آوری کمک‌های مالی | مدیران عمومی و عملیات | مدیران منابع انسانی | متخصصان منابع انسانی | متخصصان روابط کار | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | مدیران بازاریابی | مدیران برنامه‌ریزی رسانه | متخصصان روابط عمومی | استراتژیست‌های بازاریابی جستجو | مدیران خدمات اجتماعی و جامعه</t>
+          <t>مدیران خدمات اداری | نمایندگان فروش تبلیغات | مدیران تبلیغات و ترویج | تحلیلگران هوش تجاری | اساتید کسب‌وکار، پس از متوسطه | مدیران ارشد اجرایی | مدرسان ارتباطات، آموزش عالی | منشی‌های اجرایی و دستیاران اداری اجرایی | مدیران جمع‌آوری کمک‌های مالی | مدیران عمومی و عملیات | مدیران منابع انسانی | متخصصان منابع انسانی | متخصصان روابط کار | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | مدیران بازاریابی | مدیران برنامه‌ریزی رسانه | متخصصان روابط عمومی | استراتژیست‌های بازاریابی جستجو | مدیران خدمات اجتماعی و جامعه</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>صحبت کردن | تفکر انتقادی | گوش دادن فعال | درک مطلب | نوشتن | یادگیری فعال | نظارت | ریاضیات</t>
+          <t>سخن گفتن | تفکر انتقادی | گوش دادن فعال | درک مطلب | نگارش | یادگیری فعال | نظارت | ریاضیات</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -974,17 +974,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>درک شفاهی | بیان شفاهی | درک کتبی | بیان کتبی | استدلال قیاسی | وضوح گفتار | تشخیص گفتار | روانی ایده‌ها | مرتب‌سازی اطلاعات | اصالت | استدلال استقرایی | بینایی نزدیک | حساسیت به مشکل | توجه انتخابی | سهولت در اعداد | انعطاف‌پذیری دسته‌بندی</t>
+          <t>درک شفاهی | بیان شفاهی | درک کتبی | بیان کتبی | استدلال قیاسی | وضوح گفتار | تشخیص گفتار | روانی ایده‌ها | ترتیب‌دهی اطلاعات | اصالت | استدلال استقرایی | بینایی نزدیک | حساسیت به مسئله | توجه انتخابی | توانایی عددی | انعطاف‌پذیری دسته‌بندی</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ایمیل | تماس با دیگران | صرف زمان برای نشستن | فضای داخلی، با محیط کنترل‌شده | بحث‌های چهره به چهره با افراد و درون تیم‌ها | کار با یا مشارکت در یک گروه کاری یا تیم | تعیین وظایف، اولویت‌ها و اهداف | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | مکالمات تلفنی | آزادی در تصمیم‌گیری | اهمیت دقیق یا صحیح بودن | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | فرکانس تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | سطح رقابت | فشار زمانی | نامه‌ها و یادداشت‌های کتبی | پیامدهای کاری و نتایج سایر کارگران</t>
+          <t>ایمیل | ارتباط با دیگران | صرف زمان برای نشستن | محیط داخلی، دارای کنترل شرایط محیطی | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | کار با یا مشارکت در یک گروه کاری یا تیم | تعیین وظایف، اولویت‌ها و اهداف | تعامل با مشتریان خارجی یا عموم مردم | مکالمات تلفنی | آزادی در تصمیم‌گیری | اهمیت دقیق یا درست بودن | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | فراوانی تصمیم‌گیری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | سطح رقابت | فشار زمانی | نامه‌ها و یادداشت‌های کتبی | پیامدهای کاری و نتایج سایر کارکنان</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>مدیران تبلیغات و ترویج | مدیران ارشد اجرایی | مدیران جبران خدمات و مزایا | مدیران آموزش، پس از متوسطه | مصاحبه‌کنندگان واجد شرایط بودن، برنامه‌های دولتی | منشی‌های اجرایی و دستیاران اداری اجرایی | مدیران مالی | جمع‌آوری‌کنندگان کمک‌های مالی | مدیران صندوق سرمایه‌گذاری | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | مدیران بازاریابی | برنامه‌ریزان جلسه، کنوانسیون، و رویداد | مشاوران مالی شخصی | متخصصان مدیریت پروژه | مدیران روابط عمومی | متخصصان روابط عمومی | مدیران فروش | مدیران خدمات اجتماعی و جامعه | خزانه‌داران و کنترل‌کننده‌ها</t>
+          <t>مدیران تبلیغات و ترویج | مدیران ارشد اجرایی | مدیران جبران خدمات و مزایا | مدیران آموزشی، پس از متوسطه | مصاحبه‌کنندگان واجد شرایط بودن، برنامه‌های دولتی | منشی‌های اجرایی و دستیاران اداری اجرایی | مدیران مالی | جمع‌آوری‌کنندگان کمک مالی | مدیران صندوق سرمایه‌گذاری | تحلیل‌گران مدیریت | تحلیل‌گران تحقیقات بازار و متخصصان بازاریابی | مدیران بازاریابی | برنامه‌ریزان جلسات، همایش‌ها و رویدادها | مشاوران مالی شخصی | متخصصان مدیریت پروژه | مدیران روابط عمومی | متخصصان روابط عمومی | مدیران فروش | مدیران خدمات اجتماعی و جامعه | خزانه‌داران و کنترل‌کنندگان</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1016,32 +1016,32 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ADP Enterprise HR | ADP Workforce Now | Adobe Acrobat | Adobe PageMaker | Atlassian JIRA | Autodesk AutoCAD | Blackbaud The Raiser's Edge | نرم‌افزار پایگاه داده | Delphi Technology | نرم‌افزار ایمیل | FileMaker Pro | نرم‌افزار حسابداری صندوق | Google Docs | Google Drive | GroupMe | نرم‌افزار مدیریت منابع انسانی HRMS | IBM Notes | نرم‌افزار IBM Power Systems | IBM SPSS Statistics | Intuit QuickBooks | LexisNexis | LinkedIn | نرم‌افزار کدگذاری رویه پزشکی | MicroFocus GroupWise | Microsoft Access | Microsoft Dynamics | Microsoft Dynamics GP | Microsoft Excel | Microsoft Internet Explorer | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SharePoint | Microsoft Visio | Microsoft Windows XP | Microsoft Word | Minitab | Oracle Hyperion | Oracle PeopleSoft | Oracle PeopleSoft Financials | Oracle Primavera Enterprise Project Portfolio Management | PracticeWorks Systems Kodak WINOMS CS | R | SAP Business Objects | SAP BusinessObjects Crystal Reports | نرم‌افزار SAP | SAS | Sage 300 Construction and Real Estate | Sage 50 Accounting | Sage MAS 200 ERP | نرم‌افزار کنترل نظارتی و اکتساب داده SCADA | Teradata Database | نرم‌افزار مرورگر وب | نرم‌افزار Yardi</t>
+          <t>ADP Enterprise HR | ADP Workforce Now | Adobe Acrobat | Adobe PageMaker | Atlassian JIRA | Autodesk AutoCAD | Blackbaud The Raiser's Edge | نرم‌افزار پایگاه داده | Delphi Technology | نرم‌افزار ایمیل | FileMaker Pro | نرم‌افزار حسابداری صندوق | Google Docs | Google Drive | GroupMe | نرم‌افزار مدیریت منابع انسانی HRMS | IBM Notes | نرم‌افزار IBM Power Systems | IBM SPSS Statistics | Intuit QuickBooks | LexisNexis | LinkedIn | نرم‌افزار کدگذاری رویه‌های پزشکی | MicroFocus GroupWise | Microsoft Access | Microsoft Dynamics | Microsoft Dynamics GP | Microsoft Excel | Microsoft Internet Explorer | نرم‌افزار Microsoft Office | Microsoft Outlook | Microsoft PowerPoint | Microsoft Project | Microsoft Publisher | Microsoft SharePoint | Microsoft Visio | Microsoft Windows XP | Microsoft Word | Minitab | Oracle Hyperion | Oracle PeopleSoft | Oracle PeopleSoft Financials | Oracle Primavera Enterprise Project Portfolio Management | PracticeWorks Systems Kodak WINOMS CS | R | SAP Business Objects | SAP BusinessObjects Crystal Reports | نرم‌افزار SAP | SAS | Sage 300 Construction and Real Estate | Sage 50 Accounting | Sage MAS 200 ERP | نرم‌افزار کنترل نظارتی و گردآوری داده SCADA | Teradata Database | نرم‌افزار مرورگر وب | نرم‌افزار Yardi</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>گوش دادن فعال | درک مطلب | صحبت کردن | تفکر انتقادی | نوشتن | نظارت | یادگیری فعال | استراتژی‌های یادگیری</t>
+          <t>گوش دادن فعال | درک مطلب | سخن گفتن | تفکر انتقادی | نگارش | نظارت | یادگیری فعال | راهبردهای یادگیری</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>خدمات مشتری و شخصی | مدیریت و اداره | زبان انگلیسی | اداری | رایانه‌ها و الکترونیک | پرسنل و منابع انسانی | ایمنی و امنیت عمومی | ریاضیات</t>
+          <t>خدمات مشتری و شخصی | مدیریت و اداره | زبان انگلیسی | اداری | رایانه و الکترونیک | پرسنل و منابع انسانی | ایمنی و امنیت عمومی | ریاضیات</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | بینایی نزدیک | تشخیص گفتار | وضوح گفتار | استدلال قیاسی | استدلال استقرایی | حساسیت به مشکل | توجه انتخابی | انعطاف‌پذیری دسته‌بندی | مرتب‌سازی اطلاعات | روانی ایده‌ها | اشتراک زمانی | اصالت</t>
+          <t>درک شفاهی | درک کتبی | بیان شفاهی | بیان کتبی | بینایی نزدیک | تشخیص گفتار | وضوح گفتار | استدلال قیاسی | استدلال استقرایی | حساسیت به مسئله | توجه انتخابی | انعطاف‌پذیری دسته‌بندی | ترتیب‌دهی اطلاعات | روانی ایده‌ها | تقسیم توجه | اصالت</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>ایمیل | بحث‌های چهره به چهره با افراد و درون تیم‌ها | مکالمات تلفنی | کار با یا مشارکت در یک گروه کاری یا تیم | تماس با دیگران | فضای داخلی، با محیط کنترل‌شده | اهمیت دقیق یا صحیح بودن | آزادی در تصمیم‌گیری | برخورد با مشتریان خارجی یا عموم مردم به طور کلی | پیامدهای کاری و نتایج سایر کارگران | بهداشت و ایمنی سایر کارگران | تعیین وظایف، اولویت‌ها و اهداف | فرکانس تصمیم‌گیری | هماهنگی یا رهبری دیگران در انجام فعالیت‌های کاری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | فشار زمانی | صرف زمان برای نشستن | نامه‌ها و یادداشت‌های کتبی</t>
+          <t>ایمیل | گفتگوهای چهره‌به‌چهره با افراد و درون تیم‌ها | مکالمات تلفنی | کار با یا مشارکت در یک گروه کاری یا تیم | ارتباط با دیگران | محیط داخلی، دارای کنترل شرایط محیطی | اهمیت دقیق یا درست بودن | آزادی در تصمیم‌گیری | تعامل با مشتریان خارجی یا عموم مردم | پیامدهای کاری و نتایج سایر کارکنان | سلامت و ایمنی سایر کارکنان | تعیین وظایف، اولویت‌ها و اهداف | فراوانی تصمیم‌گیری | هماهنگی یا هدایت دیگران در انجام فعالیت‌های کاری | تأثیر تصمیمات بر همکاران یا نتایج شرکت | فشار زمانی | صرف زمان برای نشستن | نامه‌ها و یادداشت‌های کتبی</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>مدیران ارشد اجرایی | مدیران انطباق | متخصصان مدیریت اسناد | منشی‌های اجرایی و دستیاران اداری اجرایی | مدیران تسهیلات | سرپرستان خط اول کارگران خانه‌داری و نظافت | سرپرستان خط اول کارگران فروش غیر خرده‌فروشی | سرپرستان خط اول کارگران پشتیبانی اداری و دفتری | مدیران عمومی و عملیات | فناوران اطلاعات سلامت و ثبت‌کنندگان پزشکی | دستیاران منابع انسانی، به استثنای حقوق و دستمزد و ثبت زمان | مدیران منابع انسانی | متخصصان منابع انسانی | مدیران پروژه فناوری اطلاعات | تحلیل‌گران مدیریت | مدیران خدمات پزشکی و بهداشتی | کارمندان دفتری، عمومی | متخصصان مدیریت پروژه | منشی‌ها و دستیاران اداری، به استثنای حقوقی، پزشکی و اجرایی | مدیران خدمات اجتماعی و جامعه</t>
+          <t>مدیران ارشد اجرایی | مدیران انطباق | متخصصان مدیریت اسناد | منشی‌های اجرایی و دستیاران اداری اجرایی | مدیران تسهیلات | سرپرستان خط اول کارگران خانه‌داری و سرایداری | سرپرستان رده اول کارکنان فروش غیرخرده‌فروشی | سرپرستان خط اول کارکنان دفتری و پشتیبانی اداری | مدیران عمومی و عملیات | فن‌آوران اطلاعات سلامت و ثبت‌کنندگان پزشکی | دستیاران منابع انسانی، به جز حقوق و دستمزد و ثبت زمان | مدیران منابع انسانی | متخصصان منابع انسانی | مدیران پروژه فناوری اطلاعات | تحلیل‌گران مدیریت | مدیران خدمات پزشکی و بهداشتی | کارمندان دفتری عمومی | متخصصان مدیریت پروژه | منشی‌ها و دستیاران اداری، به جز حقوقی، پزشکی و اجرایی | مدیران خدمات اجتماعی و جامعه</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">

</xml_diff>